<commit_message>
Update supplier product master template
</commit_message>
<xml_diff>
--- a/public/templates/product-master-template.xlsx
+++ b/public/templates/product-master-template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Master" sheetId="1" r:id="R5b1622a851834ba3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup_Categories" sheetId="4" r:id="R4b45ee4d50d44ef9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup_Vehicles" sheetId="5" r:id="R3be34bf64ff84552"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup_Brands" sheetId="6" r:id="Rc6f59c225a714d4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup_Grades" sheetId="7" r:id="R0818a95c79364d17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup_SKU_Numbers" sheetId="8" r:id="Rcc0b355a1ca94fc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Expected_Results" sheetId="9" r:id="Ra41b6aa1573f446c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R97374057dedb44c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Master" sheetId="1" r:id="R991c775539b34a15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup_Categories" sheetId="2" r:id="R8dce7e882ce2464e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup_Vehicles" sheetId="3" r:id="R5a13c5570451496d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup_Brands" sheetId="4" r:id="R5271d41ad0c344b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup_Grades" sheetId="5" r:id="Rc03062f90dfa45ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup_SKU_Numbers" sheetId="6" r:id="R6d6412bd95ba43b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Expected_Results" sheetId="7" r:id="R0ed9664464b94c75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R97209a1adfc74181"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4321,7 +4321,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="81">
+  <x:cellXfs count="115">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -4511,6 +4511,102 @@
     <x:xf numFmtId="0" fontId="0" fillId="29" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="24" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="24" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="23" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -4614,7 +4710,7 @@
     <x:tableColumn id="68" name="Upload Validation | Validation Status"/>
     <x:tableColumn id="69" name="Upload Validation | Missing Fields"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
 </file>
 
@@ -4661,9 +4757,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
-        <a:ea typeface="Calibri Light"/>
-        <a:cs typeface="Calibri Light"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -5005,19 +5101,19 @@
     </x:row>
     <x:row r="2" ht="46.5" customHeight="1">
       <x:c r="A2" s="1" t="str">
-        <x:v>TATA-TIAGO-BRK-001</x:v>
+        <x:v>TOYOTA-VIN17-JACK-001</x:v>
       </x:c>
       <x:c r="B2" s="1" t="str">
-        <x:v>Tata Tiago Genuine Front Brake Pad Set</x:v>
+        <x:v>Toyota Jack Handle Extension Sub-Assembly</x:v>
       </x:c>
       <x:c r="C2" s="1" t="str">
-        <x:v>Genuine front brake pad kit for Tata Tiago and Tigor</x:v>
+        <x:v>Toyota OE jack handle extension verified against a 17VIN sample VIN</x:v>
       </x:c>
       <x:c r="D2" s="1" t="str">
-        <x:v>Genuine front brake pad kit for Tata Tiago and Tigor. Genuine Tata Tiago test inventory row.</x:v>
+        <x:v>Toyota OE part 091140G010. 17VIN returns the raw EPC name 'SUNCONJUNTO DE EXTENSION, MANIVELA DEL GATO' and marks it applicable to VIN LFMGJE720DS070251.</x:v>
       </x:c>
       <x:c r="E2" s="1" t="str">
-        <x:v>542442990107</x:v>
+        <x:v>091140G010</x:v>
       </x:c>
       <x:c r="F2" s="1" t="str">
         <x:v>Active</x:v>
@@ -5029,57 +5125,53 @@
         <x:v>New</x:v>
       </x:c>
       <x:c r="I2" s="1" t="str">
-        <x:v>TATA.1.1</x:v>
+        <x:v>TOY.2.1</x:v>
       </x:c>
       <x:c r="J2" s="1" t="str">
-        <x:v>Tiago Brake Pads</x:v>
+        <x:v>Jack Handle Extension</x:v>
       </x:c>
       <x:c r="K2" s="1" t="str">
-        <x:v>TATA.1</x:v>
+        <x:v>TOY.2</x:v>
       </x:c>
       <x:c r="L2" s="1" t="str">
         <x:v>BRD-073</x:v>
       </x:c>
       <x:c r="M2" s="1" t="str">
-        <x:v>Tata Motors</x:v>
+        <x:v>Toyota</x:v>
       </x:c>
       <x:c r="N2" s="1" t="str">
-        <x:v>Tiago Brake Pads, Tiago Oil Filters, Tiago Air Filters</x:v>
+        <x:v>Toyota OE Standard Tools</x:v>
       </x:c>
       <x:c r="O2" s="1" t="str">
-        <x:v>Tier 2</x:v>
+        <x:v>Tier 1</x:v>
       </x:c>
       <x:c r="P2" s="1" t="str">
-        <x:v>Vehicle Application</x:v>
+        <x:v>17VIN Verified VIN</x:v>
       </x:c>
       <x:c r="Q2" s="1" t="str">
-        <x:v>Tata Tiago</x:v>
+        <x:v>LFMGJE720DS070251</x:v>
       </x:c>
       <x:c r="R2" s="1"/>
       <x:c r="S2" s="1"/>
       <x:c r="T2" s="1"/>
-      <x:c r="U2" s="19" t="str">
+      <x:c r="U2" s="19" t="n">
         <x:v>216</x:v>
       </x:c>
       <x:c r="V2" s="1" t="str">
-        <x:v>Tata</x:v>
+        <x:v>Toyota</x:v>
       </x:c>
       <x:c r="W2" s="1" t="str">
-        <x:v>Tiago</x:v>
-      </x:c>
-      <x:c r="X2" s="19" t="n">
-        <x:v>2016</x:v>
-      </x:c>
-      <x:c r="Y2" s="19" t="n">
-        <x:v>2026</x:v>
-      </x:c>
+        <x:v>VIN-specific EPC record</x:v>
+      </x:c>
+      <x:c r="X2" s="19"/>
+      <x:c r="Y2" s="19"/>
       <x:c r="Z2" s="1" t="str">
-        <x:v>1.2L Petrol / 1.0L Diesel</x:v>
+        <x:v>Not provided in public 17VIN part example</x:v>
       </x:c>
       <x:c r="AA2" s="1"/>
       <x:c r="AB2" s="1"/>
       <x:c r="AC2" s="1" t="str">
-        <x:v>Confirm exact variant before fulfillment</x:v>
+        <x:v>Verified by 17VIN for VIN LFMGJE720DS070251; is_fit_for_this_vin=1; EPC applicability dates 2010-05 to 2013-11.</x:v>
       </x:c>
       <x:c r="AD2" s="20" t="n">
         <x:v>145</x:v>
@@ -5119,11 +5211,17 @@
       </x:c>
       <x:c r="AP2" s="1"/>
       <x:c r="AQ2" s="1"/>
-      <x:c r="AR2" s="1"/>
-      <x:c r="AS2" s="1"/>
-      <x:c r="AT2" s="1"/>
+      <x:c r="AR2" s="1" t="str">
+        <x:v>17VIN OE Verification</x:v>
+      </x:c>
+      <x:c r="AS2" s="1" t="str">
+        <x:v>https://en.17vin.com/doc/5106.html</x:v>
+      </x:c>
+      <x:c r="AT2" s="1" t="str">
+        <x:v>TOYOTA-VIN17-JACK-001</x:v>
+      </x:c>
       <x:c r="AU2" s="1" t="str">
-        <x:v>542442990107</x:v>
+        <x:v>091140G010</x:v>
       </x:c>
       <x:c r="AV2" s="1"/>
       <x:c r="AW2" s="1"/>
@@ -5161,19 +5259,19 @@
     </x:row>
     <x:row r="3" ht="46.5" customHeight="1">
       <x:c r="A3" s="1" t="str">
-        <x:v>TATA-TIAGO-OIL-001</x:v>
+        <x:v>TOYOTA-VIN17-WARN-001</x:v>
       </x:c>
       <x:c r="B3" s="1" t="str">
-        <x:v>Tata Tiago Genuine Engine Oil Filter</x:v>
+        <x:v>Toyota Warning Triangle Reflector Set</x:v>
       </x:c>
       <x:c r="C3" s="1" t="str">
-        <x:v>Genuine engine oil filter for Tata Tiago petrol models</x:v>
+        <x:v>Toyota OE warning triangle reflector verified against a 17VIN sample VIN</x:v>
       </x:c>
       <x:c r="D3" s="1" t="str">
-        <x:v>Genuine engine oil filter for Tata Tiago petrol models. Genuine Tata Tiago test inventory row.</x:v>
+        <x:v>Toyota OE part 8160402030. 17VIN returns the raw EPC name 'JUEGO REFLECTOR, TRIANGULO' and marks it applicable to VIN LFMGJE720DS070251.</x:v>
       </x:c>
       <x:c r="E3" s="1" t="str">
-        <x:v>571518130101</x:v>
+        <x:v>8160402030</x:v>
       </x:c>
       <x:c r="F3" s="1" t="str">
         <x:v>Active</x:v>
@@ -5185,57 +5283,53 @@
         <x:v>New</x:v>
       </x:c>
       <x:c r="I3" s="1" t="str">
-        <x:v>TATA.1.2</x:v>
+        <x:v>TOY.2.2</x:v>
       </x:c>
       <x:c r="J3" s="1" t="str">
-        <x:v>Tiago Oil Filters</x:v>
+        <x:v>Warning Triangle Reflector</x:v>
       </x:c>
       <x:c r="K3" s="1" t="str">
-        <x:v>TATA.1</x:v>
+        <x:v>TOY.2</x:v>
       </x:c>
       <x:c r="L3" s="1" t="str">
         <x:v>BRD-073</x:v>
       </x:c>
       <x:c r="M3" s="1" t="str">
-        <x:v>Tata Motors</x:v>
+        <x:v>Toyota</x:v>
       </x:c>
       <x:c r="N3" s="1" t="str">
-        <x:v>Tiago Brake Pads, Tiago Oil Filters, Tiago Air Filters</x:v>
+        <x:v>Toyota OE Safety Equipment</x:v>
       </x:c>
       <x:c r="O3" s="1" t="str">
-        <x:v>Tier 2</x:v>
+        <x:v>Tier 1</x:v>
       </x:c>
       <x:c r="P3" s="1" t="str">
-        <x:v>Vehicle Application</x:v>
+        <x:v>17VIN Verified VIN</x:v>
       </x:c>
       <x:c r="Q3" s="1" t="str">
-        <x:v>Tata Tiago</x:v>
+        <x:v>LFMGJE720DS070251</x:v>
       </x:c>
       <x:c r="R3" s="1"/>
       <x:c r="S3" s="1"/>
       <x:c r="T3" s="1"/>
-      <x:c r="U3" s="19" t="str">
+      <x:c r="U3" s="19" t="n">
         <x:v>216</x:v>
       </x:c>
       <x:c r="V3" s="1" t="str">
-        <x:v>Tata</x:v>
+        <x:v>Toyota</x:v>
       </x:c>
       <x:c r="W3" s="1" t="str">
-        <x:v>Tiago</x:v>
-      </x:c>
-      <x:c r="X3" s="19" t="n">
-        <x:v>2016</x:v>
-      </x:c>
-      <x:c r="Y3" s="19" t="n">
-        <x:v>2026</x:v>
-      </x:c>
+        <x:v>VIN-specific EPC record</x:v>
+      </x:c>
+      <x:c r="X3" s="19"/>
+      <x:c r="Y3" s="19"/>
       <x:c r="Z3" s="1" t="str">
-        <x:v>1.2L Revotron Petrol</x:v>
+        <x:v>Not provided in public 17VIN part example</x:v>
       </x:c>
       <x:c r="AA3" s="1"/>
       <x:c r="AB3" s="1"/>
       <x:c r="AC3" s="1" t="str">
-        <x:v>Confirm exact variant before fulfillment</x:v>
+        <x:v>Verified by 17VIN for VIN LFMGJE720DS070251; is_fit_for_this_vin=1; EPC applicability dates 2010-05 to 2013-11.</x:v>
       </x:c>
       <x:c r="AD3" s="20" t="n">
         <x:v>21</x:v>
@@ -5275,11 +5369,17 @@
       </x:c>
       <x:c r="AP3" s="1"/>
       <x:c r="AQ3" s="1"/>
-      <x:c r="AR3" s="1"/>
-      <x:c r="AS3" s="1"/>
-      <x:c r="AT3" s="1"/>
+      <x:c r="AR3" s="1" t="str">
+        <x:v>17VIN OE Verification</x:v>
+      </x:c>
+      <x:c r="AS3" s="1" t="str">
+        <x:v>https://en.17vin.com/doc/5105.html</x:v>
+      </x:c>
+      <x:c r="AT3" s="1" t="str">
+        <x:v>TOYOTA-VIN17-WARN-001</x:v>
+      </x:c>
       <x:c r="AU3" s="1" t="str">
-        <x:v>571518130101</x:v>
+        <x:v>8160402030</x:v>
       </x:c>
       <x:c r="AV3" s="1"/>
       <x:c r="AW3" s="1"/>
@@ -5617,7 +5717,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18e3be768b774ecd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88c7058b5cb44df9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9828,44 +9928,44 @@
     </x:row>
     <x:row r="384" ht="16.5" customHeight="1">
       <x:c r="A384" s="1" t="str">
-        <x:v>TATA.1</x:v>
+        <x:v>TOY.2</x:v>
       </x:c>
       <x:c r="B384" s="1" t="str">
-        <x:v>Tata Tiago Parts</x:v>
+        <x:v>Toyota VIN17 Verified Parts</x:v>
       </x:c>
       <x:c r="C384" s="1"/>
     </x:row>
     <x:row r="385">
       <x:c r="A385" t="str">
-        <x:v>TATA.1.1</x:v>
+        <x:v>TOY.2.1</x:v>
       </x:c>
       <x:c r="B385" t="str">
-        <x:v>Tiago Brake Pads</x:v>
+        <x:v>Jack Handle Extension</x:v>
       </x:c>
       <x:c r="C385" t="str">
-        <x:v>TATA.1</x:v>
+        <x:v>TOY.2</x:v>
       </x:c>
     </x:row>
     <x:row r="386">
       <x:c r="A386" t="str">
-        <x:v>TATA.1.2</x:v>
+        <x:v>TOY.2.2</x:v>
       </x:c>
       <x:c r="B386" t="str">
-        <x:v>Tiago Oil Filters</x:v>
+        <x:v>Warning Triangle Reflector</x:v>
       </x:c>
       <x:c r="C386" t="str">
-        <x:v>TATA.1</x:v>
+        <x:v>TOY.2</x:v>
       </x:c>
     </x:row>
     <x:row r="387">
       <x:c r="A387" t="str">
-        <x:v>TATA.1.3</x:v>
+        <x:v>TOY.2.3</x:v>
       </x:c>
       <x:c r="B387" t="str">
-        <x:v>Tiago Air Filters</x:v>
+        <x:v>Standard Tools and Safety Equipment</x:v>
       </x:c>
       <x:c r="C387" t="str">
-        <x:v>TATA.1</x:v>
+        <x:v>TOY.2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12869,31 +12969,31 @@
       <x:c r="D216" s="1"/>
     </x:row>
     <x:row r="217">
-      <x:c r="A217" t="str">
+      <x:c r="A217" t="n">
         <x:v>216</x:v>
       </x:c>
       <x:c r="B217" t="str">
-        <x:v>Tata</x:v>
+        <x:v>Toyota</x:v>
       </x:c>
       <x:c r="C217" t="str">
-        <x:v>Tiago</x:v>
+        <x:v>VIN-specific EPC record</x:v>
       </x:c>
       <x:c r="D217" t="str">
-        <x:v>Tier 2</x:v>
+        <x:v>Tier 1</x:v>
       </x:c>
     </x:row>
     <x:row r="218">
-      <x:c r="A218" t="str">
+      <x:c r="A218" t="n">
         <x:v>217</x:v>
       </x:c>
       <x:c r="B218" t="str">
-        <x:v>Tata</x:v>
+        <x:v>Toyota</x:v>
       </x:c>
       <x:c r="C218" t="str">
-        <x:v>Tiago</x:v>
+        <x:v>17VIN public API test data</x:v>
       </x:c>
       <x:c r="D218" t="str">
-        <x:v>Tier 2</x:v>
+        <x:v>Tier 1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13938,13 +14038,13 @@
         <x:v>BRD-073</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Tata Motors</x:v>
+        <x:v>Toyota</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Tiago Brake Pads, Tiago Oil Filters, Tiago Air Filters</x:v>
+        <x:v>OE Standard Tools and Safety Equipment</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Tier 2</x:v>
+        <x:v>Tier 1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14665,19 +14765,19 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B31" t="str">
-        <x:v>Tata Tiago</x:v>
+        <x:v>Toyota OE Standard Tools</x:v>
       </x:c>
       <x:c r="C31" t="str">
-        <x:v>TAT</x:v>
+        <x:v>TOY</x:v>
       </x:c>
       <x:c r="D31" t="str">
-        <x:v>Brake Pads</x:v>
+        <x:v>Jack Handle Extension</x:v>
       </x:c>
       <x:c r="E31" t="str">
-        <x:v>BRK</x:v>
+        <x:v>JHE</x:v>
       </x:c>
       <x:c r="F31" t="str">
-        <x:v>APS-TAT-BRK</x:v>
+        <x:v>APS-TOY-JHE</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -14685,60 +14785,36 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B32" t="str">
-        <x:v>Tata Tiago</x:v>
+        <x:v>Toyota OE Safety Equipment</x:v>
       </x:c>
       <x:c r="C32" t="str">
-        <x:v>TAT</x:v>
+        <x:v>TOY</x:v>
       </x:c>
       <x:c r="D32" t="str">
-        <x:v>Oil Filter</x:v>
+        <x:v>Warning Triangle Reflector</x:v>
       </x:c>
       <x:c r="E32" t="str">
-        <x:v>OIL</x:v>
+        <x:v>WTR</x:v>
       </x:c>
       <x:c r="F32" t="str">
-        <x:v>APS-TAT-OIL</x:v>
+        <x:v>APS-TOY-WTR</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B33" t="str">
-        <x:v>Tata Tiago</x:v>
-      </x:c>
-      <x:c r="C33" t="str">
-        <x:v>TAT</x:v>
-      </x:c>
-      <x:c r="D33" t="str">
-        <x:v>Petrol Air Filter</x:v>
-      </x:c>
-      <x:c r="E33" t="str">
-        <x:v>AIP</x:v>
-      </x:c>
-      <x:c r="F33" t="str">
-        <x:v>APS-TAT-AIP</x:v>
-      </x:c>
+      <x:c r="A33"/>
+      <x:c r="B33"/>
+      <x:c r="C33"/>
+      <x:c r="D33"/>
+      <x:c r="E33"/>
+      <x:c r="F33"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" t="n">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="B34" t="str">
-        <x:v>Tata Tiago</x:v>
-      </x:c>
-      <x:c r="C34" t="str">
-        <x:v>TAT</x:v>
-      </x:c>
-      <x:c r="D34" t="str">
-        <x:v>Diesel Air Filter</x:v>
-      </x:c>
-      <x:c r="E34" t="str">
-        <x:v>AID</x:v>
-      </x:c>
-      <x:c r="F34" t="str">
-        <x:v>APS-TAT-AID</x:v>
-      </x:c>
+      <x:c r="A34"/>
+      <x:c r="B34"/>
+      <x:c r="C34"/>
+      <x:c r="D34"/>
+      <x:c r="E34"/>
+      <x:c r="F34"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14759,7 +14835,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" hidden="0" customHeight="1">
       <x:c r="A1" s="68" t="str">
-        <x:v>Tata Tiago Two-Product Update Test</x:v>
+        <x:v>17VIN-Verified Toyota Two-Product Update Test</x:v>
       </x:c>
       <x:c r="B1" s="68"/>
       <x:c r="C1" s="68"/>
@@ -14769,7 +14845,7 @@
     </x:row>
     <x:row r="2" ht="26" hidden="0" customHeight="1">
       <x:c r="A2" s="69" t="str">
-        <x:v>Upload with the same supplier SKUs after the baseline upload; no duplicate products should be created.</x:v>
+        <x:v>OE/MPN and fitment are from 17VIN documentation. Prices and quantities below are test values only.</x:v>
       </x:c>
       <x:c r="B2" s="69"/>
       <x:c r="C2" s="69"/>
@@ -14807,7 +14883,7 @@
     </x:row>
     <x:row r="5" ht="36" hidden="0" customHeight="1">
       <x:c r="A5" s="71" t="str">
-        <x:v>TATA-TIAGO-BRK-001</x:v>
+        <x:v>TOYOTA-VIN17-JACK-001</x:v>
       </x:c>
       <x:c r="B5" s="72" t="str">
         <x:v>Price / Quantity Increase</x:v>
@@ -14827,7 +14903,7 @@
     </x:row>
     <x:row r="6" ht="36" hidden="0" customHeight="1">
       <x:c r="A6" s="76" t="str">
-        <x:v>TATA-TIAGO-OIL-001</x:v>
+        <x:v>TOYOTA-VIN17-WARN-001</x:v>
       </x:c>
       <x:c r="B6" s="77" t="str">
         <x:v>Price / Quantity Decrease</x:v>
@@ -14893,83 +14969,91 @@
     <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="68" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="45" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="48" t="str">
-        <x:v>Tata Tiago Part Number Sources</x:v>
-      </x:c>
-      <x:c r="B1" s="48"/>
-      <x:c r="C1" s="48"/>
-      <x:c r="D1" s="48"/>
-      <x:c r="E1" s="48"/>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="50"/>
+    <x:row r="1" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A1" s="105" t="str">
+        <x:v>17VIN-Verified Toyota EPC Sample Data</x:v>
+      </x:c>
+      <x:c r="B1" s="105"/>
+      <x:c r="C1" s="105"/>
+      <x:c r="D1" s="105"/>
+      <x:c r="E1" s="105"/>
+    </x:row>
+    <x:row r="2" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A2" s="50" t="str">
+        <x:v>The OE/MPN and VIN applicability below come from 17VIN's official API documentation. Commercial price and stock fields elsewhere in this workbook are test-only.</x:v>
+      </x:c>
       <x:c r="B2" s="50"/>
       <x:c r="C2" s="50"/>
       <x:c r="D2" s="50"/>
       <x:c r="E2" s="50"/>
     </x:row>
-    <x:row r="3" ht="24" customHeight="1">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="51" t="str">
-        <x:v>OEM Part Number</x:v>
+        <x:v>OE / MPN</x:v>
       </x:c>
       <x:c r="B3" s="51" t="str">
-        <x:v>Product</x:v>
+        <x:v>17VIN Raw Part Name</x:v>
       </x:c>
       <x:c r="C3" s="51" t="str">
-        <x:v>Vehicle</x:v>
+        <x:v>Verified VIN</x:v>
       </x:c>
       <x:c r="D3" s="51" t="str">
-        <x:v>Source URL</x:v>
+        <x:v>Official 17VIN Source URL</x:v>
       </x:c>
       <x:c r="E3" s="51" t="str">
-        <x:v>VIN Test Result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="42" customHeight="1">
+        <x:v>Verification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A4" s="52" t="str">
-        <x:v>OEM 542442990107</x:v>
+        <x:v>091140G010</x:v>
       </x:c>
       <x:c r="B4" s="53" t="str">
-        <x:v>Front Brake Pad Set</x:v>
+        <x:v>SUNCONJUNTO DE EXTENSION, MANIVELA DEL GATO</x:v>
       </x:c>
       <x:c r="C4" s="53" t="str">
-        <x:v>Tata Tiago / Tigor</x:v>
+        <x:v>LFMGJE720DS070251</x:v>
       </x:c>
       <x:c r="D4" s="53" t="str">
-        <x:v>https://mechdeals.com/product-detail/kit-pad-66484</x:v>
+        <x:v>https://en.17vin.com/doc/5106.html</x:v>
       </x:c>
       <x:c r="E4" s="56" t="str">
-        <x:v>17VIN routing error 1006</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="42" customHeight="1">
+        <x:v>partnumber_original matches; is_fit_for_this_vin=1; begin 201005; end 201311</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A5" s="57" t="str">
-        <x:v>OEM 571518130101</x:v>
+        <x:v>8160402030</x:v>
       </x:c>
       <x:c r="B5" s="58" t="str">
-        <x:v>Engine Oil Filter</x:v>
+        <x:v>JUEGO REFLECTOR, TRIANGULO</x:v>
       </x:c>
       <x:c r="C5" s="58" t="str">
-        <x:v>Tata Tiago petrol</x:v>
+        <x:v>LFMGJE720DS070251</x:v>
       </x:c>
       <x:c r="D5" s="58" t="str">
-        <x:v>https://mechdeals.com/product-detail/oil-filter-assy-37457</x:v>
+        <x:v>https://en.17vin.com/doc/5105.html</x:v>
       </x:c>
       <x:c r="E5" s="61" t="str">
-        <x:v>17VIN routing error 1006</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="42" customHeight="1">
+        <x:v>partnumber_original matches; is_fit_for_this_vin=1; begin 201005; end 201311</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A6" s="57"/>
-      <x:c r="B6" s="58"/>
+      <x:c r="B6" s="58" t="str">
+        <x:v>English product names in Product_Master are readable translations of the raw 17VIN EPC names.</x:v>
+      </x:c>
       <x:c r="C6" s="58"/>
-      <x:c r="D6" s="58"/>
-      <x:c r="E6" s="61"/>
+      <x:c r="D6" s="58" t="str">
+        <x:v>https://en.17vin.com/doc.html</x:v>
+      </x:c>
+      <x:c r="E6" s="61" t="str">
+        <x:v>No unsupported engine, transmission, trim or exact model has been invented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="63"/>

</xml_diff>